<commit_message>
feat(permisos): consolidar a 5 grupos finales (15 checkboxes)
Antes: 7 grupos. Ahora: 5 grupos por simplicidad operativa.

Mapeo definitivo:
- centro_control: centro_control
- operaciones: logistica, envios, devoluciones, incidencias, historico,
               b2b, contraentrega, inventario
- finanzas: finanzas
- comercial: comercial, revenue, inteligencia
- configuracion: configuracion, usuarios, auditoria

Contraentrega e Inventario ahora viven dentro de Operaciones porque
ambos son flujos logisticos (stock + fulfillment + COD).
</commit_message>
<xml_diff>
--- a/sheets/Produccion_Sheet_Plantilla.xlsx
+++ b/sheets/Produccion_Sheet_Plantilla.xlsx
@@ -486,7 +486,7 @@
     <t xml:space="preserve">COSTO TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">PRECIO SUGERIDO DE VENTA</t>
+    <t xml:space="preserve">PRECIO SUGERIDO DE VENTA (CON IVA)</t>
   </si>
   <si>
     <t xml:space="preserve">Costo base (sin IVA)</t>
@@ -495,13 +495,13 @@
     <t xml:space="preserve">Margen %</t>
   </si>
   <si>
+    <t xml:space="preserve">PRECIO VENTA (con IVA)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Precio antes de IVA</t>
   </si>
   <si>
     <t xml:space="preserve">IVA 19%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Precio final con IVA</t>
   </si>
   <si>
     <t xml:space="preserve">Margen real %</t>
@@ -658,7 +658,7 @@
     <numFmt numFmtId="169" formatCode="0%"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -830,6 +830,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF666666"/>
@@ -970,7 +977,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1059,15 +1066,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1079,59 +1082,59 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1151,7 +1154,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1161,10 +1164,6 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2192,13 +2191,13 @@
   <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2212,773 +2211,801 @@
       <c r="F1" s="20"/>
       <c r="G1" s="20"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="8" t="s">
         <v>88</v>
       </c>
       <c r="C2" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="23"/>
+      <c r="E2" s="22"/>
       <c r="F2" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="G2" s="22"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="8" t="s">
         <v>93</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="8" t="s">
         <v>95</v>
       </c>
       <c r="F3" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="G3" s="23" t="n">
         <v>0.19</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="24" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="9" t="n">
         <v>15900</v>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="27" t="n">
         <f aca="false">ROUND(F6*$G$3,0)</f>
         <v>3021</v>
       </c>
-      <c r="F6" s="30" t="n">
+      <c r="F6" s="27" t="n">
         <f aca="false">C6*D6</f>
         <v>15900</v>
       </c>
-      <c r="G6" s="30" t="n">
+      <c r="G6" s="27" t="n">
         <f aca="false">F6+E6</f>
         <v>18921</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26"/>
-      <c r="B7" s="27" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="25"/>
+      <c r="B7" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="27" t="n">
         <f aca="false">ROUND(F7*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="27" t="n">
         <f aca="false">C7*D7</f>
         <v>0</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="27" t="n">
         <f aca="false">F7+E7</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="9" t="n">
         <v>15900</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="10" t="n">
         <v>1.07</v>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="27" t="n">
         <f aca="false">ROUND(F8*$G$3,0)</f>
         <v>3232</v>
       </c>
-      <c r="F8" s="30" t="n">
+      <c r="F8" s="27" t="n">
         <f aca="false">C8*D8</f>
         <v>17013</v>
       </c>
-      <c r="G8" s="30" t="n">
+      <c r="G8" s="27" t="n">
         <f aca="false">F8+E8</f>
         <v>20245</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26"/>
-      <c r="B9" s="27" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="25"/>
+      <c r="B9" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="9" t="n">
         <v>4400</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="10" t="n">
         <v>0.15</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E9" s="27" t="n">
         <f aca="false">ROUND(F9*$G$3,0)</f>
         <v>125</v>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="F9" s="27" t="n">
         <f aca="false">C9*D9</f>
         <v>660</v>
       </c>
-      <c r="G9" s="30" t="n">
+      <c r="G9" s="27" t="n">
         <f aca="false">F9+E9</f>
         <v>785</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26"/>
-      <c r="B10" s="27" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="25"/>
+      <c r="B10" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="27" t="n">
         <f aca="false">ROUND(F10*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="30" t="n">
+      <c r="F10" s="27" t="n">
         <f aca="false">C10*D10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="30" t="n">
+      <c r="G10" s="27" t="n">
         <f aca="false">F10+E10</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="E11" s="27" t="n">
         <f aca="false">ROUND(F11*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="30" t="n">
+      <c r="F11" s="27" t="n">
         <f aca="false">C11*D11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="30" t="n">
+      <c r="G11" s="27" t="n">
         <f aca="false">F11+E11</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="26"/>
-      <c r="B12" s="27" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="25"/>
+      <c r="B12" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="9" t="n">
         <v>1200</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="27" t="n">
         <f aca="false">ROUND(F12*$G$3,0)</f>
         <v>228</v>
       </c>
-      <c r="F12" s="30" t="n">
+      <c r="F12" s="27" t="n">
         <f aca="false">C12*D12</f>
         <v>1200</v>
       </c>
-      <c r="G12" s="30" t="n">
+      <c r="G12" s="27" t="n">
         <f aca="false">F12+E12</f>
         <v>1428</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="26" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="9" t="n">
         <v>10700</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="30" t="n">
+      <c r="E13" s="27" t="n">
         <f aca="false">ROUND(F13*$G$3,0)</f>
         <v>2033</v>
       </c>
-      <c r="F13" s="30" t="n">
+      <c r="F13" s="27" t="n">
         <f aca="false">C13*D13</f>
         <v>10700</v>
       </c>
-      <c r="G13" s="30" t="n">
+      <c r="G13" s="27" t="n">
         <f aca="false">F13+E13</f>
         <v>12733</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="25" t="s">
         <v>115</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="26" t="s">
         <v>116</v>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="D14" s="29" t="n">
+      <c r="D14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="30" t="n">
+      <c r="E14" s="27" t="n">
         <f aca="false">ROUND(F14*$G$3,0)</f>
         <v>133</v>
       </c>
-      <c r="F14" s="30" t="n">
+      <c r="F14" s="27" t="n">
         <f aca="false">C14*D14</f>
         <v>700</v>
       </c>
-      <c r="G14" s="30" t="n">
+      <c r="G14" s="27" t="n">
         <f aca="false">F14+E14</f>
         <v>833</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26"/>
-      <c r="B15" s="27" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="25"/>
+      <c r="B15" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="9" t="n">
         <v>87</v>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="27" t="n">
         <f aca="false">ROUND(F15*$G$3,0)</f>
         <v>17</v>
       </c>
-      <c r="F15" s="30" t="n">
+      <c r="F15" s="27" t="n">
         <f aca="false">C15*D15</f>
         <v>87</v>
       </c>
-      <c r="G15" s="30" t="n">
+      <c r="G15" s="27" t="n">
         <f aca="false">F15+E15</f>
         <v>104</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="25"/>
+      <c r="B16" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="29" t="n">
+      <c r="D16" s="10" t="n">
         <v>0.07</v>
       </c>
-      <c r="E16" s="30" t="n">
+      <c r="E16" s="27" t="n">
         <f aca="false">ROUND(F16*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="30" t="n">
+      <c r="F16" s="27" t="n">
         <f aca="false">C16*D16</f>
         <v>0</v>
       </c>
-      <c r="G16" s="30" t="n">
+      <c r="G16" s="27" t="n">
         <f aca="false">F16+E16</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="28" t="n">
+      <c r="C17" s="9" t="n">
         <v>7000</v>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="30" t="n">
+      <c r="E17" s="27" t="n">
         <f aca="false">ROUND(F17*$G$3,0)</f>
         <v>1330</v>
       </c>
-      <c r="F17" s="30" t="n">
+      <c r="F17" s="27" t="n">
         <f aca="false">C17*D17</f>
         <v>7000</v>
       </c>
-      <c r="G17" s="30" t="n">
+      <c r="G17" s="27" t="n">
         <f aca="false">F17+E17</f>
         <v>8330</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="26"/>
-      <c r="B18" s="27" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="25"/>
+      <c r="B18" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="C18" s="28" t="n">
+      <c r="C18" s="9" t="n">
         <v>2100</v>
       </c>
-      <c r="D18" s="29" t="n">
+      <c r="D18" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="30" t="n">
+      <c r="E18" s="27" t="n">
         <f aca="false">ROUND(F18*$G$3,0)</f>
         <v>399</v>
       </c>
-      <c r="F18" s="30" t="n">
+      <c r="F18" s="27" t="n">
         <f aca="false">C18*D18</f>
         <v>2100</v>
       </c>
-      <c r="G18" s="30" t="n">
+      <c r="G18" s="27" t="n">
         <f aca="false">F18+E18</f>
         <v>2499</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="26" t="s">
+      <c r="A19" s="25" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="C19" s="28" t="n">
+      <c r="C19" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="E19" s="27" t="n">
         <f aca="false">ROUND(F19*$G$3,0)</f>
         <v>4</v>
       </c>
-      <c r="F19" s="30" t="n">
+      <c r="F19" s="27" t="n">
         <f aca="false">C19*D19</f>
         <v>20</v>
       </c>
-      <c r="G19" s="30" t="n">
+      <c r="G19" s="27" t="n">
         <f aca="false">F19+E19</f>
         <v>24</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="25"/>
+      <c r="B20" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="C20" s="28" t="n">
+      <c r="C20" s="9" t="n">
         <v>123</v>
       </c>
-      <c r="D20" s="29" t="n">
+      <c r="D20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="30" t="n">
+      <c r="E20" s="27" t="n">
         <f aca="false">ROUND(F20*$G$3,0)</f>
         <v>23</v>
       </c>
-      <c r="F20" s="30" t="n">
+      <c r="F20" s="27" t="n">
         <f aca="false">C20*D20</f>
         <v>123</v>
       </c>
-      <c r="G20" s="30" t="n">
+      <c r="G20" s="27" t="n">
         <f aca="false">F20+E20</f>
         <v>146</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="26"/>
-      <c r="B21" s="27" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="25"/>
+      <c r="B21" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="C21" s="28" t="n">
+      <c r="C21" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="D21" s="29" t="n">
+      <c r="D21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="30" t="n">
+      <c r="E21" s="27" t="n">
         <f aca="false">ROUND(F21*$G$3,0)</f>
         <v>2</v>
       </c>
-      <c r="F21" s="30" t="n">
+      <c r="F21" s="27" t="n">
         <f aca="false">C21*D21</f>
         <v>10</v>
       </c>
-      <c r="G21" s="30" t="n">
+      <c r="G21" s="27" t="n">
         <f aca="false">F21+E21</f>
         <v>12</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="25"/>
+      <c r="B22" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="C22" s="28" t="n">
+      <c r="C22" s="9" t="n">
         <v>180</v>
       </c>
-      <c r="D22" s="29" t="n">
+      <c r="D22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="30" t="n">
+      <c r="E22" s="27" t="n">
         <f aca="false">ROUND(F22*$G$3,0)</f>
         <v>34</v>
       </c>
-      <c r="F22" s="30" t="n">
+      <c r="F22" s="27" t="n">
         <f aca="false">C22*D22</f>
         <v>180</v>
       </c>
-      <c r="G22" s="30" t="n">
+      <c r="G22" s="27" t="n">
         <f aca="false">F22+E22</f>
         <v>214</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
+      <c r="A23" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="27" t="s">
+      <c r="B23" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="C23" s="28" t="n">
+      <c r="C23" s="9" t="n">
         <v>278</v>
       </c>
-      <c r="D23" s="29" t="n">
+      <c r="D23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="30" t="n">
+      <c r="E23" s="27" t="n">
         <f aca="false">ROUND(F23*$G$3,0)</f>
         <v>53</v>
       </c>
-      <c r="F23" s="30" t="n">
+      <c r="F23" s="27" t="n">
         <f aca="false">C23*D23</f>
         <v>278</v>
       </c>
-      <c r="G23" s="30" t="n">
+      <c r="G23" s="27" t="n">
         <f aca="false">F23+E23</f>
         <v>331</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25"/>
+      <c r="B24" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="C24" s="28" t="n">
+      <c r="C24" s="9" t="n">
         <v>111</v>
       </c>
-      <c r="D24" s="29" t="n">
+      <c r="D24" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="30" t="n">
+      <c r="E24" s="27" t="n">
         <f aca="false">ROUND(F24*$G$3,0)</f>
         <v>42</v>
       </c>
-      <c r="F24" s="30" t="n">
+      <c r="F24" s="27" t="n">
         <f aca="false">C24*D24</f>
         <v>222</v>
       </c>
-      <c r="G24" s="30" t="n">
+      <c r="G24" s="27" t="n">
         <f aca="false">F24+E24</f>
         <v>264</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26"/>
-      <c r="B25" s="27" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="25"/>
+      <c r="B25" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="C25" s="28" t="n">
+      <c r="C25" s="9" t="n">
         <v>700</v>
       </c>
-      <c r="D25" s="29" t="n">
+      <c r="D25" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="30" t="n">
+      <c r="E25" s="27" t="n">
         <f aca="false">ROUND(F25*$G$3,0)</f>
         <v>133</v>
       </c>
-      <c r="F25" s="30" t="n">
+      <c r="F25" s="27" t="n">
         <f aca="false">C25*D25</f>
         <v>700</v>
       </c>
-      <c r="G25" s="30" t="n">
+      <c r="G25" s="27" t="n">
         <f aca="false">F25+E25</f>
         <v>833</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="26"/>
-      <c r="B26" s="27" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="25"/>
+      <c r="B26" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="C26" s="28" t="n">
+      <c r="C26" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="29" t="n">
+      <c r="D26" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="30" t="n">
+      <c r="E26" s="27" t="n">
         <f aca="false">ROUND(F26*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="30" t="n">
+      <c r="F26" s="27" t="n">
         <f aca="false">C26*D26</f>
         <v>0</v>
       </c>
-      <c r="G26" s="30" t="n">
+      <c r="G26" s="27" t="n">
         <f aca="false">F26+E26</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26"/>
-      <c r="B27" s="27" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="25"/>
+      <c r="B27" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="C27" s="28" t="n">
+      <c r="C27" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="29" t="n">
+      <c r="D27" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="30" t="n">
+      <c r="E27" s="27" t="n">
         <f aca="false">ROUND(F27*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="30" t="n">
+      <c r="F27" s="27" t="n">
         <f aca="false">C27*D27</f>
         <v>0</v>
       </c>
-      <c r="G27" s="30" t="n">
+      <c r="G27" s="27" t="n">
         <f aca="false">F27+E27</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="26" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="B28" s="27" t="s">
+      <c r="B28" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="C28" s="28" t="n">
+      <c r="C28" s="9" t="n">
         <v>11000</v>
       </c>
-      <c r="D28" s="29" t="n">
+      <c r="D28" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="30" t="n">
+      <c r="E28" s="27" t="n">
         <f aca="false">ROUND(F28*$G$3,0)</f>
         <v>2090</v>
       </c>
-      <c r="F28" s="30" t="n">
+      <c r="F28" s="27" t="n">
         <f aca="false">C28*D28</f>
         <v>11000</v>
       </c>
-      <c r="G28" s="30" t="n">
+      <c r="G28" s="27" t="n">
         <f aca="false">F28+E28</f>
         <v>13090</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="31"/>
-      <c r="B29" s="32" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="28"/>
+      <c r="B29" s="29" t="s">
         <v>133</v>
       </c>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="33" t="n">
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="30" t="n">
         <f aca="false">SUM(F6:F28)</f>
         <v>67893</v>
       </c>
-      <c r="G29" s="33" t="n">
+      <c r="G29" s="30" t="n">
         <f aca="false">SUM(G6:G28)</f>
         <v>80792</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="34" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="31" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B32" s="35" t="n">
+      <c r="B32" s="33" t="n">
         <f aca="false">F29</f>
         <v>67893</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+    </row>
+    <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="B33" s="25" t="s">
+      <c r="B33" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="C33" s="25" t="s">
+      <c r="C33" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="D33" s="25" t="s">
+      <c r="D33" s="24" t="s">
         <v>139</v>
       </c>
-      <c r="E33" s="25" t="s">
+      <c r="E33" s="24" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="24" t="n">
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="23" t="n">
         <v>0.5</v>
       </c>
-      <c r="B34" s="30" t="n">
-        <f aca="false">ROUND($B$32*(1+A34),0)</f>
-        <v>101840</v>
-      </c>
-      <c r="C34" s="30" t="n">
-        <f aca="false">ROUND(B34*$G$3,0)</f>
+      <c r="B34" s="34" t="n">
+        <f aca="false">ROUND($B$32*(1+A34)*(1+$G$3),0)</f>
+        <v>121189</v>
+      </c>
+      <c r="C34" s="35" t="n">
+        <f aca="false">ROUND(B34/(1+$G$3),0)</f>
+        <v>101839</v>
+      </c>
+      <c r="D34" s="34" t="n">
+        <f aca="false">B34-C34</f>
         <v>19350</v>
       </c>
-      <c r="D34" s="36" t="n">
-        <f aca="false">B34+C34</f>
-        <v>121190</v>
-      </c>
-      <c r="E34" s="37" t="n">
-        <f aca="false">IF(B34=0,0,(B34-$B$32)/B34)</f>
-        <v>0.333336606441477</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="24" t="n">
+      <c r="E34" s="36" t="n">
+        <f aca="false">IF(C34=0,0,(C34-$B$32)/C34)</f>
+        <v>0.33333006019305</v>
+      </c>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="23" t="n">
         <v>0.65</v>
       </c>
-      <c r="B35" s="30" t="n">
-        <f aca="false">ROUND($B$32*(1+A35),0)</f>
-        <v>112023</v>
-      </c>
-      <c r="C35" s="30" t="n">
-        <f aca="false">ROUND(B35*$G$3,0)</f>
+      <c r="B35" s="34" t="n">
+        <f aca="false">ROUND($B$32*(1+A35)*(1+$G$3),0)</f>
+        <v>133308</v>
+      </c>
+      <c r="C35" s="35" t="n">
+        <f aca="false">ROUND(B35/(1+$G$3),0)</f>
+        <v>112024</v>
+      </c>
+      <c r="D35" s="34" t="n">
+        <f aca="false">B35-C35</f>
         <v>21284</v>
       </c>
-      <c r="D35" s="36" t="n">
-        <f aca="false">B35+C35</f>
-        <v>133307</v>
-      </c>
-      <c r="E35" s="37" t="n">
-        <f aca="false">IF(B35=0,0,(B35-$B$32)/B35)</f>
-        <v>0.393936959374414</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="24" t="n">
+      <c r="E35" s="36" t="n">
+        <f aca="false">IF(C35=0,0,(C35-$B$32)/C35)</f>
+        <v>0.393942369492252</v>
+      </c>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="23" t="n">
         <v>0.8</v>
       </c>
-      <c r="B36" s="30" t="n">
-        <f aca="false">ROUND($B$32*(1+A36),0)</f>
-        <v>122207</v>
-      </c>
-      <c r="C36" s="30" t="n">
-        <f aca="false">ROUND(B36*$G$3,0)</f>
+      <c r="B36" s="34" t="n">
+        <f aca="false">ROUND($B$32*(1+A36)*(1+$G$3),0)</f>
+        <v>145427</v>
+      </c>
+      <c r="C36" s="35" t="n">
+        <f aca="false">ROUND(B36/(1+$G$3),0)</f>
+        <v>122208</v>
+      </c>
+      <c r="D36" s="34" t="n">
+        <f aca="false">B36-C36</f>
         <v>23219</v>
       </c>
-      <c r="D36" s="36" t="n">
-        <f aca="false">B36+C36</f>
-        <v>145426</v>
-      </c>
-      <c r="E36" s="37" t="n">
-        <f aca="false">IF(B36=0,0,(B36-$B$32)/B36)</f>
-        <v>0.444442626036152</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E36" s="36" t="n">
+        <f aca="false">IF(C36=0,0,(C36-$B$32)/C36)</f>
+        <v>0.444447172034564</v>
+      </c>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="32"/>
+      <c r="B37" s="32"/>
+      <c r="C37" s="32"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+    </row>
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B38" s="22"/>
+      <c r="B38" s="8"/>
       <c r="C38" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="D38" s="22"/>
+      <c r="D38" s="8"/>
       <c r="F38" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="G38" s="22"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="38" t="s">
+      <c r="G38" s="8"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="37" t="s">
         <v>144</v>
       </c>
-      <c r="B40" s="38"/>
-      <c r="C40" s="38"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="38"/>
-      <c r="F40" s="38"/>
-      <c r="G40" s="38"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="37"/>
+      <c r="E40" s="37"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -3057,7 +3084,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="38" t="s">
         <v>154</v>
       </c>
     </row>
@@ -3095,14 +3122,14 @@
       <c r="F1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="39" t="s">
         <v>156</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
@@ -3128,13 +3155,13 @@
       <c r="A6" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="40" t="s">
         <v>47</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D6" s="42" t="n">
+      <c r="D6" s="41" t="n">
         <f aca="false">IFERROR(VLOOKUP(B6,Inventario!$A$7:$E$20,5,0),0)</f>
         <v>69</v>
       </c>
@@ -3151,58 +3178,58 @@
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="42" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="44" t="s">
+      <c r="A10" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="44" t="s">
+      <c r="C10" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="44" t="s">
+      <c r="D10" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="44" t="s">
+      <c r="E10" s="43" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="45"/>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45"/>
+      <c r="A11" s="44"/>
+      <c r="B11" s="44"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="45"/>
-      <c r="B12" s="45"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
+      <c r="A12" s="44"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="45"/>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="45"/>
+      <c r="A13" s="44"/>
+      <c r="B13" s="44"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="45"/>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
+      <c r="A14" s="44"/>
+      <c r="B14" s="44"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="43" t="s">
+      <c r="A16" s="42" t="s">
         <v>166</v>
       </c>
     </row>
@@ -3248,81 +3275,81 @@
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="42" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="44" t="s">
+      <c r="A23" s="43" t="s">
         <v>176</v>
       </c>
-      <c r="B23" s="44" t="s">
+      <c r="B23" s="43" t="s">
         <v>177</v>
       </c>
-      <c r="C23" s="44" t="s">
+      <c r="C23" s="43" t="s">
         <v>178</v>
       </c>
-      <c r="D23" s="44" t="s">
+      <c r="D23" s="43" t="s">
         <v>179</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E23" s="43" t="s">
         <v>180</v>
       </c>
-      <c r="F23" s="44" t="s">
+      <c r="F23" s="43" t="s">
         <v>181</v>
       </c>
-      <c r="G23" s="44" t="s">
+      <c r="G23" s="43" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="46"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
+      <c r="A24" s="45"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="43" t="s">
+      <c r="A26" s="42" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="47" t="s">
+      <c r="A27" s="46" t="s">
         <v>184</v>
       </c>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
+      <c r="B27" s="46"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="47"/>
-      <c r="B28" s="47"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="47"/>
+      <c r="A28" s="46"/>
+      <c r="B28" s="46"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="47"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="47"/>
+      <c r="A29" s="46"/>
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="B31" s="48"/>
-      <c r="C31" s="48"/>
+      <c r="B31" s="22"/>
+      <c r="C31" s="22"/>
       <c r="D31" s="21" t="s">
         <v>186</v>
       </c>

</xml_diff>

<commit_message>
fix(auth): capturar y devolver error real en PATCH /usuarios
Antes los 500 en PATCH /usuarios/:id se devolvian sin CORS headers, por
lo que el navegador los reportaba como CORS error y no se veia el
mensaje real. Ahora capturamos cualquier excepcion, la logueamos a
stdout (visible en Railway logs) y la devolvemos como HTTPException
con detail visible al cliente.

Esto nos permite diagnosticar por que el guardar de permisos falla.
</commit_message>
<xml_diff>
--- a/sheets/Produccion_Sheet_Plantilla.xlsx
+++ b/sheets/Produccion_Sheet_Plantilla.xlsx
@@ -82,9 +82,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="187">
-  <si>
-    <t xml:space="preserve">MALE'DENIM OS — Plantilla de Producción (Fase 1)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="183">
+  <si>
+    <t xml:space="preserve">Plantilla de Producción — Fase 1</t>
   </si>
   <si>
     <t xml:space="preserve">Hojas conectadas con fórmulas para mostrar la mecánica del módulo.</t>
@@ -93,7 +93,7 @@
     <t xml:space="preserve">1) Órdenes de Ingreso</t>
   </si>
   <si>
-    <t xml:space="preserve">Transcribe la hoja de la textilera, un renglón por rollo. Columnas grises (código/barcode) las genera el sistema.</t>
+    <t xml:space="preserve">Transcribe la hoja de la textilera, un renglón por rollo. Columnas en azul acero (código/barcode) las genera el sistema.</t>
   </si>
   <si>
     <t xml:space="preserve">2) Inventario</t>
@@ -111,13 +111,13 @@
     <t xml:space="preserve">4) Precosteo (formato)</t>
   </si>
   <si>
-    <t xml:space="preserve">Espejo de tu formato 14500-1: líneas por categoría con IVA, costo total y precio sugerido. Al firmar se archiva en Histórico y se limpia.</t>
+    <t xml:space="preserve">Espejo de tu formato: líneas por categoría con IVA, costo total y precio sugerido (con IVA). Al firmar se archiva en Histórico y se limpia.</t>
   </si>
   <si>
     <t xml:space="preserve">5) Histórico Precosteo</t>
   </si>
   <si>
-    <t xml:space="preserve">Donde quedan archivados los precosteos firmados (lo llena el botón Guardar y firmar).</t>
+    <t xml:space="preserve">Donde quedan archivados los precosteos firmados.</t>
   </si>
   <si>
     <t xml:space="preserve">6) Orden de Corte (formato)</t>
@@ -126,31 +126,19 @@
     <t xml:space="preserve">Documento que da luz verde al cortador.</t>
   </si>
   <si>
+    <t xml:space="preserve">Marca</t>
+  </si>
+  <si>
     <t xml:space="preserve">Colores</t>
   </si>
   <si>
-    <t xml:space="preserve">Encabezado azul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lo llenas tú.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Encabezado gris</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lo llena el sistema.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Texto azul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ejemplos — bórralos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guardar y limpiar (reset a 0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En Google Sheets se activa con el script Apps Script adjunto: archiva el formato en Histórico y deja los campos en 0. En el módulo es automático.</t>
+    <t xml:space="preserve">DEEP INK #213033 · GRAPHITE #606060 · STEEL BLUE #87A6B8 · SOFT CONCRETE #E1E1DF · acentos cream/teal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipografía</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montserrat (equivalente de Gotham). Texto editable en azul #0C457A.</t>
   </si>
   <si>
     <t xml:space="preserve">textilera</t>
@@ -297,7 +285,7 @@
     <t xml:space="preserve">BRUSELAS INDIGO 9.8oz</t>
   </si>
   <si>
-    <t xml:space="preserve">INVENTARIO DE TELA — unificado por nombre</t>
+    <t xml:space="preserve">          INVENTARIO DE TELA — unificado por nombre</t>
   </si>
   <si>
     <t xml:space="preserve">Ver tela:</t>
@@ -342,7 +330,7 @@
     <t xml:space="preserve">Cortador 1</t>
   </si>
   <si>
-    <t xml:space="preserve">PRECOSTEO · MALE'DENIM OS</t>
+    <t xml:space="preserve">          PRECOSTEO</t>
   </si>
   <si>
     <t xml:space="preserve">REF</t>
@@ -540,7 +528,7 @@
     <t xml:space="preserve">costo_total_con_iva</t>
   </si>
   <si>
-    <t xml:space="preserve">precio_sugerido</t>
+    <t xml:space="preserve">precio_venta_con_iva</t>
   </si>
   <si>
     <t xml:space="preserve">autorizado_por</t>
@@ -549,7 +537,7 @@
     <t xml:space="preserve">(las filas firmadas se agregan aquí automáticamente)</t>
   </si>
   <si>
-    <t xml:space="preserve">ORDEN DE CORTE · MALE'DENIM OS</t>
+    <t xml:space="preserve">          ORDEN DE CORTE</t>
   </si>
   <si>
     <t xml:space="preserve">Documento que autoriza al cortador a iniciar (luz verde)</t>
@@ -658,7 +646,7 @@
     <numFmt numFmtId="169" formatCode="0%"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -683,30 +671,24 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FF1F3A5F"/>
-      <name val="Arial"/>
+      <sz val="15"/>
+      <color rgb="FF213033"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
+      <color rgb="FF213033"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF2E5A88"/>
-      <name val="Arial"/>
+      <color rgb="FF213033"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -714,21 +696,21 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
+      <color rgb="FF0C457A"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <color rgb="FF213033"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -739,54 +721,48 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="15"/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
+      <color rgb="FF0C457A"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="12"/>
-      <color rgb="FF1E7A46"/>
-      <name val="Arial"/>
+      <color rgb="FF036A73"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF1E7A46"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <color rgb="FF036A73"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF2E5A88"/>
-      <name val="Arial"/>
+      <color rgb="FF036A73"/>
+      <name val="Montserrat"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF213033"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -794,22 +770,22 @@
       <b val="true"/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
+      <color rgb="FF606060"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
+      <color rgb="FF213033"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -817,30 +793,15 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF1F3A5F"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF333333"/>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <i val="true"/>
       <sz val="9"/>
-      <color rgb="FF666666"/>
-      <name val="Arial"/>
+      <color rgb="FF606060"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -848,14 +809,14 @@
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF999999"/>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
+      <color rgb="FF0C457A"/>
+      <name val="Montserrat"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -869,38 +830,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3A5F"/>
-        <bgColor rgb="FF333333"/>
+        <fgColor rgb="FF213033"/>
+        <bgColor rgb="FF333300"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF8A94A6"/>
+        <fgColor rgb="FF87A6B8"/>
         <bgColor rgb="FF999999"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2F7"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFF2F1EF"/>
+        <bgColor rgb="FFF1EAD8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF6CC"/>
-        <bgColor rgb="FFEEF2F7"/>
+        <fgColor rgb="FFF1EAD8"/>
+        <bgColor rgb="FFF2F1EF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E5A88"/>
-        <bgColor rgb="FF1F3A5F"/>
+        <fgColor rgb="FF606060"/>
+        <bgColor rgb="FF808080"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDCE5EF"/>
-        <bgColor rgb="FFEEF2F7"/>
+        <fgColor rgb="FFE1E1DF"/>
+        <bgColor rgb="FFF1EAD8"/>
       </patternFill>
     </fill>
   </fills>
@@ -977,192 +938,180 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1190,13 +1139,13 @@
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF1E7A46"/>
+      <rgbColor rgb="FF036A73"/>
       <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF8A94A6"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF87A6B8"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF6CC"/>
-      <rgbColor rgb="FFEEF2F7"/>
+      <rgbColor rgb="FFF2F1EF"/>
+      <rgbColor rgb="FFE1E1DF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1210,8 +1159,8 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFDCE5EF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFF1EAD8"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -1223,19 +1172,148 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666666"/>
+      <rgbColor rgb="FF606060"/>
       <rgbColor rgb="FF999999"/>
-      <rgbColor rgb="FF1F3A5F"/>
+      <rgbColor rgb="FF0C457A"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF2E5A88"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF213033"/>
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1638000</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>171360</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1638000" cy="552240"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>676080</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>228240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="676080" cy="228240"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>732960</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>247320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="732960" cy="247320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1418,124 +1496,104 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A4:B18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="92"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="4" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2"/>
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2"/>
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2"/>
+      <c r="B15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1546,6 +1604,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1557,288 +1616,288 @@
   <dimension ref="A1:P6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="M1" s="6" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="G2" s="7"/>
+      <c r="H2" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="I2" s="7"/>
+      <c r="J2" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="K2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8" t="s">
+      <c r="M2" s="9" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="N2" s="8" t="n">
+        <v>9800</v>
+      </c>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8" t="s">
+      <c r="G3" s="7"/>
+      <c r="H3" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>9800</v>
+      </c>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="M2" s="10" t="n">
-        <v>47.9</v>
-      </c>
-      <c r="N2" s="9" t="n">
-        <v>9800</v>
-      </c>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8" t="s">
+      <c r="E4" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>82</v>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>12500</v>
+      </c>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="C5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="M3" s="10" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="N3" s="9" t="n">
-        <v>9800</v>
-      </c>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="D5" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="8" t="s">
+      <c r="F5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="I5" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="J5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="K5" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="H4" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="J4" s="8" t="s">
+      <c r="L5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>80.1</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>12500</v>
+      </c>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="L4" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="M4" s="10" t="n">
-        <v>82</v>
-      </c>
-      <c r="N4" s="9" t="n">
-        <v>12500</v>
-      </c>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="M5" s="10" t="n">
-        <v>80.1</v>
-      </c>
-      <c r="N5" s="9" t="n">
-        <v>12500</v>
-      </c>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="K6" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="M6" s="10" t="n">
+      <c r="L6" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="M6" s="9" t="n">
         <v>307.7</v>
       </c>
-      <c r="N6" s="9" t="n">
+      <c r="N6" s="8" t="n">
         <v>16000</v>
       </c>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -1866,71 +1925,71 @@
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3" s="14" t="n">
+    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="13" t="n">
         <f aca="false">IFERROR(VLOOKUP(B3,$A$7:$E$20,2,0),0)</f>
         <v>2</v>
       </c>
-      <c r="E3" s="15" t="str">
+      <c r="E3" s="14" t="str">
         <f aca="false">IFERROR("Disponible: "&amp;TEXT(VLOOKUP(B3,$A$7:$E$20,5,0),"#,##0.0")&amp;" m","")</f>
         <v>Disponible: 69.0 m</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="17" t="n">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="16" t="n">
         <f aca="false">IF($A7="","",COUNTIF('Órdenes de Ingreso'!$K:$K,$A7))</f>
         <v>2</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="17" t="n">
         <f aca="false">IF($A7="","",SUMIF('Órdenes de Ingreso'!$K:$K,$A7,'Órdenes de Ingreso'!$M:$M))</f>
         <v>99</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">IF($A7="","",SUMIF(Cortes!$B:$B,$A7,Cortes!$D:$D))</f>
         <v>30</v>
       </c>
@@ -1939,19 +1998,19 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="17" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="16" t="n">
         <f aca="false">IF($A8="","",COUNTIF('Órdenes de Ingreso'!$K:$K,$A8))</f>
         <v>2</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="17" t="n">
         <f aca="false">IF($A8="","",SUMIF('Órdenes de Ingreso'!$K:$K,$A8,'Órdenes de Ingreso'!$M:$M))</f>
         <v>162.1</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">IF($A8="","",SUMIF(Cortes!$B:$B,$A8,Cortes!$D:$D))</f>
         <v>0</v>
       </c>
@@ -1960,19 +2019,19 @@
         <v>162.1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" s="17" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="16" t="n">
         <f aca="false">IF($A9="","",COUNTIF('Órdenes de Ingreso'!$K:$K,$A9))</f>
         <v>1</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="17" t="n">
         <f aca="false">IF($A9="","",SUMIF('Órdenes de Ingreso'!$K:$K,$A9,'Órdenes de Ingreso'!$M:$M))</f>
         <v>307.7</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="17" t="n">
         <f aca="false">IF($A9="","",SUMIF(Cortes!$B:$B,$A9,Cortes!$D:$D))</f>
         <v>0</v>
       </c>
@@ -1981,17 +2040,17 @@
         <v>307.7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
-      <c r="B10" s="17" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7"/>
+      <c r="B10" s="16" t="str">
         <f aca="false">IF($A10="","",COUNTIF('Órdenes de Ingreso'!$K:$K,$A10))</f>
         <v/>
       </c>
-      <c r="C10" s="18" t="str">
+      <c r="C10" s="17" t="str">
         <f aca="false">IF($A10="","",SUMIF('Órdenes de Ingreso'!$K:$K,$A10,'Órdenes de Ingreso'!$M:$M))</f>
         <v/>
       </c>
-      <c r="D10" s="18" t="str">
+      <c r="D10" s="17" t="str">
         <f aca="false">IF($A10="","",SUMIF(Cortes!$B:$B,$A10,Cortes!$D:$D))</f>
         <v/>
       </c>
@@ -2000,17 +2059,17 @@
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
-      <c r="B11" s="17" t="str">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7"/>
+      <c r="B11" s="16" t="str">
         <f aca="false">IF($A11="","",COUNTIF('Órdenes de Ingreso'!$K:$K,$A11))</f>
         <v/>
       </c>
-      <c r="C11" s="18" t="str">
+      <c r="C11" s="17" t="str">
         <f aca="false">IF($A11="","",SUMIF('Órdenes de Ingreso'!$K:$K,$A11,'Órdenes de Ingreso'!$M:$M))</f>
         <v/>
       </c>
-      <c r="D11" s="18" t="str">
+      <c r="D11" s="17" t="str">
         <f aca="false">IF($A11="","",SUMIF(Cortes!$B:$B,$A11,Cortes!$D:$D))</f>
         <v/>
       </c>
@@ -2047,123 +2106,123 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="B2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>84</v>
       </c>
       <c r="D2" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
       <c r="D3" s="19"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
       <c r="D4" s="19"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
       <c r="D5" s="19"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
       <c r="D6" s="19"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
       <c r="D7" s="19"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
       <c r="D8" s="19"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
       <c r="D9" s="19"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
       <c r="D10" s="19"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
       <c r="D11" s="19"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2191,821 +2250,793 @@
   <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="E2" s="21"/>
+      <c r="F2" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="B3" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="C3" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="22"/>
-      <c r="F2" s="21" t="s">
+      <c r="D3" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G2" s="8"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="21" t="s">
+      <c r="F3" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="G3" s="22" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="B5" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="C5" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="D5" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="G3" s="23" t="n">
-        <v>0.19</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+      <c r="E5" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="F5" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="G5" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="D5" s="24" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="B6" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="F5" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="G5" s="24" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="8" t="n">
         <v>15900</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="27" t="n">
+      <c r="E6" s="26" t="n">
         <f aca="false">ROUND(F6*$G$3,0)</f>
         <v>3021</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="26" t="n">
         <f aca="false">C6*D6</f>
         <v>15900</v>
       </c>
-      <c r="G6" s="27" t="n">
+      <c r="G6" s="26" t="n">
         <f aca="false">F6+E6</f>
         <v>18921</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25"/>
-      <c r="B7" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" s="9" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24"/>
+      <c r="B7" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="27" t="n">
+      <c r="E7" s="26" t="n">
         <f aca="false">ROUND(F7*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="27" t="n">
+      <c r="F7" s="26" t="n">
         <f aca="false">C7*D7</f>
         <v>0</v>
       </c>
-      <c r="G7" s="27" t="n">
+      <c r="G7" s="26" t="n">
         <f aca="false">F7+E7</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="C8" s="9" t="n">
+      <c r="A8" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="8" t="n">
         <v>15900</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="9" t="n">
         <v>1.07</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="26" t="n">
         <f aca="false">ROUND(F8*$G$3,0)</f>
         <v>3232</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="26" t="n">
         <f aca="false">C8*D8</f>
         <v>17013</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="26" t="n">
         <f aca="false">F8+E8</f>
         <v>20245</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25"/>
-      <c r="B9" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="9" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24"/>
+      <c r="B9" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="8" t="n">
         <v>4400</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="9" t="n">
         <v>0.15</v>
       </c>
-      <c r="E9" s="27" t="n">
+      <c r="E9" s="26" t="n">
         <f aca="false">ROUND(F9*$G$3,0)</f>
         <v>125</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="26" t="n">
         <f aca="false">C9*D9</f>
         <v>660</v>
       </c>
-      <c r="G9" s="27" t="n">
+      <c r="G9" s="26" t="n">
         <f aca="false">F9+E9</f>
         <v>785</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25"/>
-      <c r="B10" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" s="9" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24"/>
+      <c r="B10" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="27" t="n">
+      <c r="E10" s="26" t="n">
         <f aca="false">ROUND(F10*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="26" t="n">
         <f aca="false">C10*D10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="27" t="n">
+      <c r="G10" s="26" t="n">
         <f aca="false">F10+E10</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>110</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="9" t="n">
+      <c r="A11" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="27" t="n">
+      <c r="E11" s="26" t="n">
         <f aca="false">ROUND(F11*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">C11*D11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="26" t="n">
         <f aca="false">F11+E11</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25"/>
-      <c r="B12" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="C12" s="9" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24"/>
+      <c r="B12" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="8" t="n">
         <v>1200</v>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="D12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="27" t="n">
+      <c r="E12" s="26" t="n">
         <f aca="false">ROUND(F12*$G$3,0)</f>
         <v>228</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="26" t="n">
         <f aca="false">C12*D12</f>
         <v>1200</v>
       </c>
-      <c r="G12" s="27" t="n">
+      <c r="G12" s="26" t="n">
         <f aca="false">F12+E12</f>
         <v>1428</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="26" t="s">
-        <v>114</v>
-      </c>
-      <c r="C13" s="9" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" s="8" t="n">
         <v>10700</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="27" t="n">
+      <c r="E13" s="26" t="n">
         <f aca="false">ROUND(F13*$G$3,0)</f>
         <v>2033</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="26" t="n">
         <f aca="false">C13*D13</f>
         <v>10700</v>
       </c>
-      <c r="G13" s="27" t="n">
+      <c r="G13" s="26" t="n">
         <f aca="false">F13+E13</f>
         <v>12733</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="C14" s="9" t="n">
+      <c r="A14" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" s="8" t="n">
         <v>700</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="27" t="n">
+      <c r="E14" s="26" t="n">
         <f aca="false">ROUND(F14*$G$3,0)</f>
         <v>133</v>
       </c>
-      <c r="F14" s="27" t="n">
+      <c r="F14" s="26" t="n">
         <f aca="false">C14*D14</f>
         <v>700</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="26" t="n">
         <f aca="false">F14+E14</f>
         <v>833</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25"/>
-      <c r="B15" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="C15" s="9" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24"/>
+      <c r="B15" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="8" t="n">
         <v>87</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="27" t="n">
+      <c r="E15" s="26" t="n">
         <f aca="false">ROUND(F15*$G$3,0)</f>
         <v>17</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="26" t="n">
         <f aca="false">C15*D15</f>
         <v>87</v>
       </c>
-      <c r="G15" s="27" t="n">
+      <c r="G15" s="26" t="n">
         <f aca="false">F15+E15</f>
         <v>104</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25"/>
-      <c r="B16" s="26" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" s="9" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24"/>
+      <c r="B16" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D16" s="9" t="n">
         <v>0.07</v>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="26" t="n">
         <f aca="false">ROUND(F16*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="26" t="n">
         <f aca="false">C16*D16</f>
         <v>0</v>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="26" t="n">
         <f aca="false">F16+E16</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="B17" s="26" t="s">
-        <v>119</v>
-      </c>
-      <c r="C17" s="9" t="n">
+      <c r="A17" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" s="8" t="n">
         <v>7000</v>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="27" t="n">
+      <c r="E17" s="26" t="n">
         <f aca="false">ROUND(F17*$G$3,0)</f>
         <v>1330</v>
       </c>
-      <c r="F17" s="27" t="n">
+      <c r="F17" s="26" t="n">
         <f aca="false">C17*D17</f>
         <v>7000</v>
       </c>
-      <c r="G17" s="27" t="n">
+      <c r="G17" s="26" t="n">
         <f aca="false">F17+E17</f>
         <v>8330</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25"/>
-      <c r="B18" s="26" t="s">
-        <v>120</v>
-      </c>
-      <c r="C18" s="9" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24"/>
+      <c r="B18" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="C18" s="8" t="n">
         <v>2100</v>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="27" t="n">
+      <c r="E18" s="26" t="n">
         <f aca="false">ROUND(F18*$G$3,0)</f>
         <v>399</v>
       </c>
-      <c r="F18" s="27" t="n">
+      <c r="F18" s="26" t="n">
         <f aca="false">C18*D18</f>
         <v>2100</v>
       </c>
-      <c r="G18" s="27" t="n">
+      <c r="G18" s="26" t="n">
         <f aca="false">F18+E18</f>
         <v>2499</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
-        <v>121</v>
-      </c>
-      <c r="B19" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="C19" s="9" t="n">
+      <c r="A19" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E19" s="26" t="n">
         <f aca="false">ROUND(F19*$G$3,0)</f>
         <v>4</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="26" t="n">
         <f aca="false">C19*D19</f>
         <v>20</v>
       </c>
-      <c r="G19" s="27" t="n">
+      <c r="G19" s="26" t="n">
         <f aca="false">F19+E19</f>
         <v>24</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25"/>
-      <c r="B20" s="26" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24"/>
+      <c r="B20" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" s="8" t="n">
         <v>123</v>
       </c>
-      <c r="C20" s="9" t="n">
-        <v>123</v>
-      </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="27" t="n">
+      <c r="E20" s="26" t="n">
         <f aca="false">ROUND(F20*$G$3,0)</f>
         <v>23</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="26" t="n">
         <f aca="false">C20*D20</f>
         <v>123</v>
       </c>
-      <c r="G20" s="27" t="n">
+      <c r="G20" s="26" t="n">
         <f aca="false">F20+E20</f>
         <v>146</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25"/>
-      <c r="B21" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="C21" s="9" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24"/>
+      <c r="B21" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="C21" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E21" s="26" t="n">
         <f aca="false">ROUND(F21*$G$3,0)</f>
         <v>2</v>
       </c>
-      <c r="F21" s="27" t="n">
+      <c r="F21" s="26" t="n">
         <f aca="false">C21*D21</f>
         <v>10</v>
       </c>
-      <c r="G21" s="27" t="n">
+      <c r="G21" s="26" t="n">
         <f aca="false">F21+E21</f>
         <v>12</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="25"/>
-      <c r="B22" s="26" t="s">
-        <v>125</v>
-      </c>
-      <c r="C22" s="9" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24"/>
+      <c r="B22" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="C22" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="D22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="27" t="n">
+      <c r="E22" s="26" t="n">
         <f aca="false">ROUND(F22*$G$3,0)</f>
         <v>34</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="26" t="n">
         <f aca="false">C22*D22</f>
         <v>180</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="26" t="n">
         <f aca="false">F22+E22</f>
         <v>214</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
-        <v>126</v>
-      </c>
-      <c r="B23" s="26" t="s">
-        <v>127</v>
-      </c>
-      <c r="C23" s="9" t="n">
+      <c r="A23" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="8" t="n">
         <v>278</v>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D23" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="27" t="n">
+      <c r="E23" s="26" t="n">
         <f aca="false">ROUND(F23*$G$3,0)</f>
         <v>53</v>
       </c>
-      <c r="F23" s="27" t="n">
+      <c r="F23" s="26" t="n">
         <f aca="false">C23*D23</f>
         <v>278</v>
       </c>
-      <c r="G23" s="27" t="n">
+      <c r="G23" s="26" t="n">
         <f aca="false">F23+E23</f>
         <v>331</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25"/>
-      <c r="B24" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="C24" s="9" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="24"/>
+      <c r="B24" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" s="8" t="n">
         <v>111</v>
       </c>
-      <c r="D24" s="10" t="n">
+      <c r="D24" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="27" t="n">
+      <c r="E24" s="26" t="n">
         <f aca="false">ROUND(F24*$G$3,0)</f>
         <v>42</v>
       </c>
-      <c r="F24" s="27" t="n">
+      <c r="F24" s="26" t="n">
         <f aca="false">C24*D24</f>
         <v>222</v>
       </c>
-      <c r="G24" s="27" t="n">
+      <c r="G24" s="26" t="n">
         <f aca="false">F24+E24</f>
         <v>264</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25"/>
-      <c r="B25" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="C25" s="9" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="24"/>
+      <c r="B25" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" s="8" t="n">
         <v>700</v>
       </c>
-      <c r="D25" s="10" t="n">
+      <c r="D25" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="27" t="n">
+      <c r="E25" s="26" t="n">
         <f aca="false">ROUND(F25*$G$3,0)</f>
         <v>133</v>
       </c>
-      <c r="F25" s="27" t="n">
+      <c r="F25" s="26" t="n">
         <f aca="false">C25*D25</f>
         <v>700</v>
       </c>
-      <c r="G25" s="27" t="n">
+      <c r="G25" s="26" t="n">
         <f aca="false">F25+E25</f>
         <v>833</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25"/>
-      <c r="B26" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="C26" s="9" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="24"/>
+      <c r="B26" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="10" t="n">
+      <c r="D26" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="27" t="n">
+      <c r="E26" s="26" t="n">
         <f aca="false">ROUND(F26*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="27" t="n">
+      <c r="F26" s="26" t="n">
         <f aca="false">C26*D26</f>
         <v>0</v>
       </c>
-      <c r="G26" s="27" t="n">
+      <c r="G26" s="26" t="n">
         <f aca="false">F26+E26</f>
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25"/>
-      <c r="B27" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="C27" s="9" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="24"/>
+      <c r="B27" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="C27" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="10" t="n">
+      <c r="D27" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="27" t="n">
+      <c r="E27" s="26" t="n">
         <f aca="false">ROUND(F27*$G$3,0)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="27" t="n">
+      <c r="F27" s="26" t="n">
         <f aca="false">C27*D27</f>
         <v>0</v>
       </c>
-      <c r="G27" s="27" t="n">
+      <c r="G27" s="26" t="n">
         <f aca="false">F27+E27</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
-        <v>132</v>
-      </c>
-      <c r="B28" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="C28" s="9" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="B28" s="25" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" s="8" t="n">
         <v>11000</v>
       </c>
-      <c r="D28" s="10" t="n">
+      <c r="D28" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="27" t="n">
+      <c r="E28" s="26" t="n">
         <f aca="false">ROUND(F28*$G$3,0)</f>
         <v>2090</v>
       </c>
-      <c r="F28" s="27" t="n">
+      <c r="F28" s="26" t="n">
         <f aca="false">C28*D28</f>
         <v>11000</v>
       </c>
-      <c r="G28" s="27" t="n">
+      <c r="G28" s="26" t="n">
         <f aca="false">F28+E28</f>
         <v>13090</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28"/>
-      <c r="B29" s="29" t="s">
-        <v>133</v>
-      </c>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="30" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="27"/>
+      <c r="B29" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="C29" s="27"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="29" t="n">
         <f aca="false">SUM(F6:F28)</f>
         <v>67893</v>
       </c>
-      <c r="G29" s="30" t="n">
+      <c r="G29" s="29" t="n">
         <f aca="false">SUM(G6:G28)</f>
         <v>80792</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="31" t="s">
-        <v>134</v>
-      </c>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="B32" s="33" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="B32" s="30" t="n">
         <f aca="false">F29</f>
         <v>67893</v>
       </c>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
-    </row>
-    <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="24" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B33" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="E33" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="B33" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="C33" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="D33" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="E33" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23" t="n">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="B34" s="34" t="n">
+      <c r="B34" s="31" t="n">
         <f aca="false">ROUND($B$32*(1+A34)*(1+$G$3),0)</f>
         <v>121189</v>
       </c>
-      <c r="C34" s="35" t="n">
+      <c r="C34" s="32" t="n">
         <f aca="false">ROUND(B34/(1+$G$3),0)</f>
         <v>101839</v>
       </c>
-      <c r="D34" s="34" t="n">
+      <c r="D34" s="33" t="n">
         <f aca="false">B34-C34</f>
         <v>19350</v>
       </c>
-      <c r="E34" s="36" t="n">
+      <c r="E34" s="34" t="n">
         <f aca="false">IF(C34=0,0,(C34-$B$32)/C34)</f>
         <v>0.33333006019305</v>
       </c>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="23" t="n">
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="22" t="n">
         <v>0.65</v>
       </c>
-      <c r="B35" s="34" t="n">
+      <c r="B35" s="31" t="n">
         <f aca="false">ROUND($B$32*(1+A35)*(1+$G$3),0)</f>
         <v>133308</v>
       </c>
-      <c r="C35" s="35" t="n">
+      <c r="C35" s="32" t="n">
         <f aca="false">ROUND(B35/(1+$G$3),0)</f>
         <v>112024</v>
       </c>
-      <c r="D35" s="34" t="n">
+      <c r="D35" s="33" t="n">
         <f aca="false">B35-C35</f>
         <v>21284</v>
       </c>
-      <c r="E35" s="36" t="n">
+      <c r="E35" s="34" t="n">
         <f aca="false">IF(C35=0,0,(C35-$B$32)/C35)</f>
         <v>0.393942369492252</v>
       </c>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="23" t="n">
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="n">
         <v>0.8</v>
       </c>
-      <c r="B36" s="34" t="n">
+      <c r="B36" s="31" t="n">
         <f aca="false">ROUND($B$32*(1+A36)*(1+$G$3),0)</f>
         <v>145427</v>
       </c>
-      <c r="C36" s="35" t="n">
+      <c r="C36" s="32" t="n">
         <f aca="false">ROUND(B36/(1+$G$3),0)</f>
         <v>122208</v>
       </c>
-      <c r="D36" s="34" t="n">
+      <c r="D36" s="33" t="n">
         <f aca="false">B36-C36</f>
         <v>23219</v>
       </c>
-      <c r="E36" s="36" t="n">
+      <c r="E36" s="34" t="n">
         <f aca="false">IF(C36=0,0,(C36-$B$32)/C36)</f>
         <v>0.444447172034564</v>
       </c>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="32"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-    </row>
-    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="21" t="s">
-        <v>141</v>
-      </c>
-      <c r="B38" s="8"/>
-      <c r="C38" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="D38" s="8"/>
-      <c r="F38" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="G38" s="8"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="37" t="s">
-        <v>144</v>
-      </c>
-      <c r="B40" s="37"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="37"/>
-      <c r="F40" s="37"/>
-      <c r="G40" s="37"/>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="B38" s="7"/>
+      <c r="C38" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="F38" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="G38" s="7"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="B40" s="35"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="35"/>
+      <c r="E40" s="35"/>
+      <c r="F40" s="35"/>
+      <c r="G40" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -3033,6 +3064,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3044,48 +3076,47 @@
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F1" s="6" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="36" t="s">
         <v>150</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38" t="s">
-        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3107,253 +3138,253 @@
   <dimension ref="A1:G31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="39" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-    </row>
-    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="21" t="s">
+      <c r="B6" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="D4" s="8"/>
-    </row>
-    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
-        <v>159</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="21" t="s">
-        <v>160</v>
-      </c>
-      <c r="D5" s="8"/>
-    </row>
-    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>161</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="D6" s="41" t="n">
+      <c r="D6" s="39" t="n">
         <f aca="false">IFERROR(VLOOKUP(B6,Inventario!$A$7:$E$20,5,0),0)</f>
         <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="D7" s="8"/>
+      <c r="A7" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="D7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="42" t="s">
-        <v>165</v>
+      <c r="A9" s="4" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="43" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="43" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="43" t="s">
-        <v>81</v>
+      <c r="A10" s="40" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="40" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44"/>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
+      <c r="A11" s="41"/>
+      <c r="B11" s="41"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44"/>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="44"/>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
+      <c r="A13" s="41"/>
+      <c r="B13" s="41"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="44"/>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
+      <c r="A14" s="41"/>
+      <c r="B14" s="41"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="41"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="4" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="20" t="s">
+        <v>164</v>
+      </c>
+      <c r="D17" s="7"/>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18" s="20" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="20" t="s">
         <v>167</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="21" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="D17" s="8"/>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
+      <c r="D19" s="7"/>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="20" t="s">
         <v>169</v>
       </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="21" t="s">
+      <c r="B20" s="7"/>
+      <c r="C20" s="20" t="s">
         <v>170</v>
       </c>
-      <c r="D18" s="8"/>
-    </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="D19" s="8"/>
-    </row>
-    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>173</v>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="7"/>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="40" t="s">
+        <v>172</v>
+      </c>
+      <c r="B23" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="C23" s="40" t="s">
+        <v>174</v>
+      </c>
+      <c r="D23" s="40" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="43" t="s">
+      <c r="E23" s="40" t="s">
         <v>176</v>
       </c>
-      <c r="B23" s="43" t="s">
+      <c r="F23" s="40" t="s">
         <v>177</v>
       </c>
-      <c r="C23" s="43" t="s">
+      <c r="G23" s="40" t="s">
         <v>178</v>
       </c>
-      <c r="D23" s="43" t="s">
-        <v>179</v>
-      </c>
-      <c r="E23" s="43" t="s">
-        <v>180</v>
-      </c>
-      <c r="F23" s="43" t="s">
-        <v>181</v>
-      </c>
-      <c r="G23" s="43" t="s">
-        <v>182</v>
-      </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="45"/>
-      <c r="B24" s="45"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
+      <c r="G24" s="42"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="42" t="s">
-        <v>183</v>
+      <c r="A26" s="4" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="46" t="s">
-        <v>184</v>
-      </c>
-      <c r="B27" s="46"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="46"/>
-      <c r="E27" s="46"/>
-      <c r="F27" s="46"/>
+      <c r="A27" s="43" t="s">
+        <v>180</v>
+      </c>
+      <c r="B27" s="43"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="46"/>
-      <c r="B28" s="46"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
+      <c r="A28" s="43"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="46"/>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
+      <c r="A29" s="43"/>
+      <c r="B29" s="43"/>
+      <c r="C29" s="43"/>
+      <c r="D29" s="43"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="s">
-        <v>185</v>
-      </c>
-      <c r="B31" s="22"/>
-      <c r="C31" s="22"/>
-      <c r="D31" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="E31" s="8"/>
+      <c r="A31" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="E31" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3379,5 +3410,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>